<commit_message>
updates to formatting of test files as requested in other PRs
</commit_message>
<xml_diff>
--- a/rules/CORE-000068/negative/01/data/unit-test-coreid-CG0641-negative.xlsx
+++ b/rules/CORE-000068/negative/01/data/unit-test-coreid-CG0641-negative.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marisa_wyckmans\CORE\CDISC_Rule_Authoring\core-contributor\rules\CORE-000068\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A620875-6607-4210-A4F8-20619A41520A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00D824C7-E9CB-4843-AE4E-ED21B42B0BE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21240" windowHeight="15270" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="79">
   <si>
     <t>Product</t>
   </si>
@@ -257,51 +257,6 @@
   </si>
   <si>
     <t>Drug A</t>
-  </si>
-  <si>
-    <t>ABC12301002</t>
-  </si>
-  <si>
-    <t>NOT HISPANIC OR LATINO</t>
-  </si>
-  <si>
-    <t>P</t>
-  </si>
-  <si>
-    <t>Placebo</t>
-  </si>
-  <si>
-    <t>ABC12301003</t>
-  </si>
-  <si>
-    <t>F</t>
-  </si>
-  <si>
-    <t>BLACK OR AFRICAN AMERICAN</t>
-  </si>
-  <si>
-    <t>ABC12301004</t>
-  </si>
-  <si>
-    <t>ASIAN</t>
-  </si>
-  <si>
-    <t>SCREEN FAILURE</t>
-  </si>
-  <si>
-    <t>ABC12302001</t>
-  </si>
-  <si>
-    <t>GONZALEZ, E</t>
-  </si>
-  <si>
-    <t>AMERICAN INDIAN OR ALASKA NATIVE</t>
-  </si>
-  <si>
-    <t>ABC12302002</t>
-  </si>
-  <si>
-    <t>NATIVE HAWAIIAN OR OTHER PACIFIC ISLANDERS</t>
   </si>
   <si>
     <t>[PRESENT]</t>
@@ -338,7 +293,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -355,12 +310,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor rgb="FFFFFFCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEDEDED"/>
-        <bgColor rgb="FFEDEDED"/>
       </patternFill>
     </fill>
   </fills>
@@ -406,7 +355,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -415,23 +364,13 @@
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -828,7 +767,7 @@
         <v>28</v>
       </c>
       <c r="F2" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -838,10 +777,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:AG16"/>
+  <dimension ref="A1:Z5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>14</v>
       </c>
@@ -920,676 +859,314 @@
       <c r="Z1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="AA1" s="4"/>
-      <c r="AB1" s="4"/>
-      <c r="AC1" s="4"/>
-      <c r="AD1" s="4"/>
-      <c r="AE1" s="4"/>
-      <c r="AF1" s="4"/>
-      <c r="AG1" s="4"/>
     </row>
-    <row r="2" spans="1:33" ht="90" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:26" ht="90" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="K2" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="L2" s="5" t="s">
+      <c r="K2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="L2" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="M2" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="N2" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="O2" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="P2" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="Q2" s="5" t="s">
+      <c r="Q2" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="R2" s="5" t="s">
+      <c r="R2" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="S2" s="5" t="s">
+      <c r="S2" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="T2" s="5" t="s">
+      <c r="T2" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="U2" s="5" t="s">
+      <c r="U2" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="V2" s="5" t="s">
+      <c r="V2" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="W2" s="5" t="s">
+      <c r="W2" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="X2" s="5" t="s">
+      <c r="X2" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="Y2" s="5" t="s">
+      <c r="Y2" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="Z2" s="5" t="s">
+      <c r="Z2" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="AA2" s="6"/>
-      <c r="AB2" s="6"/>
-      <c r="AC2" s="6"/>
-      <c r="AD2" s="6"/>
-      <c r="AE2" s="6"/>
-      <c r="AF2" s="6"/>
-      <c r="AG2" s="6"/>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="L3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="M3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="N3" s="5" t="s">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="N3" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="O3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="P3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="R3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="S3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="T3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="U3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="V3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="W3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="X3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="Y3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="Z3" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="AA3" s="7"/>
-      <c r="AB3" s="7"/>
-      <c r="AC3" s="7"/>
-      <c r="AD3" s="7"/>
-      <c r="AE3" s="7"/>
-      <c r="AF3" s="7"/>
-      <c r="AG3" s="7"/>
+      <c r="O3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="S3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="T3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="U3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="V3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="W3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="X3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="Y3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="Z3" s="4" t="s">
+        <v>66</v>
+      </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A4" s="5">
-        <v>50</v>
-      </c>
-      <c r="B4" s="5">
-        <v>50</v>
-      </c>
-      <c r="C4" s="5">
-        <v>50</v>
-      </c>
-      <c r="D4" s="5">
-        <v>50</v>
-      </c>
-      <c r="E4" s="5">
-        <v>50</v>
-      </c>
-      <c r="F4" s="5">
-        <v>50</v>
-      </c>
-      <c r="G4" s="5">
-        <v>50</v>
-      </c>
-      <c r="H4" s="5">
-        <v>50</v>
-      </c>
-      <c r="I4" s="5">
-        <v>50</v>
-      </c>
-      <c r="J4" s="5">
-        <v>50</v>
-      </c>
-      <c r="K4" s="5">
-        <v>50</v>
-      </c>
-      <c r="L4" s="5">
-        <v>50</v>
-      </c>
-      <c r="M4" s="5">
-        <v>50</v>
-      </c>
-      <c r="N4" s="5">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
+        <v>50</v>
+      </c>
+      <c r="B4" s="4">
+        <v>50</v>
+      </c>
+      <c r="C4" s="4">
+        <v>50</v>
+      </c>
+      <c r="D4" s="4">
+        <v>50</v>
+      </c>
+      <c r="E4" s="4">
+        <v>50</v>
+      </c>
+      <c r="F4" s="4">
+        <v>50</v>
+      </c>
+      <c r="G4" s="4">
+        <v>50</v>
+      </c>
+      <c r="H4" s="4">
+        <v>50</v>
+      </c>
+      <c r="I4" s="4">
+        <v>50</v>
+      </c>
+      <c r="J4" s="4">
+        <v>50</v>
+      </c>
+      <c r="K4" s="4">
+        <v>50</v>
+      </c>
+      <c r="L4" s="4">
+        <v>50</v>
+      </c>
+      <c r="M4" s="4">
+        <v>50</v>
+      </c>
+      <c r="N4" s="4">
         <v>8</v>
       </c>
-      <c r="O4" s="5">
-        <v>50</v>
-      </c>
-      <c r="P4" s="5">
-        <v>50</v>
-      </c>
-      <c r="Q4" s="5">
-        <v>50</v>
-      </c>
-      <c r="R4" s="5">
-        <v>50</v>
-      </c>
-      <c r="S4" s="5">
-        <v>50</v>
-      </c>
-      <c r="T4" s="5">
-        <v>50</v>
-      </c>
-      <c r="U4" s="5">
-        <v>50</v>
-      </c>
-      <c r="V4" s="5">
-        <v>50</v>
-      </c>
-      <c r="W4" s="5">
-        <v>50</v>
-      </c>
-      <c r="X4" s="5">
-        <v>50</v>
-      </c>
-      <c r="Y4" s="5">
-        <v>50</v>
-      </c>
-      <c r="Z4" s="5">
-        <v>50</v>
-      </c>
-      <c r="AA4" s="7"/>
-      <c r="AB4" s="7"/>
-      <c r="AC4" s="7"/>
-      <c r="AD4" s="7"/>
-      <c r="AE4" s="7"/>
-      <c r="AF4" s="7"/>
-      <c r="AG4" s="7"/>
+      <c r="O4" s="4">
+        <v>50</v>
+      </c>
+      <c r="P4" s="4">
+        <v>50</v>
+      </c>
+      <c r="Q4" s="4">
+        <v>50</v>
+      </c>
+      <c r="R4" s="4">
+        <v>50</v>
+      </c>
+      <c r="S4" s="4">
+        <v>50</v>
+      </c>
+      <c r="T4" s="4">
+        <v>50</v>
+      </c>
+      <c r="U4" s="4">
+        <v>50</v>
+      </c>
+      <c r="V4" s="4">
+        <v>50</v>
+      </c>
+      <c r="W4" s="4">
+        <v>50</v>
+      </c>
+      <c r="X4" s="4">
+        <v>50</v>
+      </c>
+      <c r="Y4" s="4">
+        <v>50</v>
+      </c>
+      <c r="Z4" s="4">
+        <v>50</v>
+      </c>
     </row>
-    <row r="5" spans="1:33" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+    <row r="5" spans="1:26" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="5">
         <v>1001</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="6">
         <v>38729</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="6">
         <v>38786</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="6">
         <v>38729</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="6">
         <v>38786</v>
       </c>
-      <c r="I5" s="9">
+      <c r="I5" s="6">
         <v>38720</v>
       </c>
-      <c r="J5" s="9">
+      <c r="J5" s="6">
         <v>38808</v>
       </c>
-      <c r="K5" s="8">
+      <c r="K5" s="5">
         <v>1</v>
       </c>
-      <c r="L5" s="8" t="s">
+      <c r="L5" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="M5" s="8">
+      <c r="M5" s="5">
         <v>17880</v>
       </c>
-      <c r="N5" s="8">
+      <c r="N5" s="5">
         <v>57</v>
       </c>
-      <c r="P5" s="8" t="s">
+      <c r="P5" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="Q5" s="8" t="s">
+      <c r="Q5" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="R5" s="8" t="s">
+      <c r="R5" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="S5" s="8" t="s">
+      <c r="S5" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="T5" s="8" t="s">
+      <c r="T5" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="U5" s="8" t="s">
+      <c r="U5" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="V5" s="8" t="s">
+      <c r="V5" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="W5" s="8" t="s">
+      <c r="W5" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="AA5" s="10"/>
-      <c r="AB5" s="10"/>
-      <c r="AC5" s="10"/>
-      <c r="AD5" s="10"/>
-      <c r="AE5" s="10"/>
-      <c r="AF5" s="10"/>
-      <c r="AG5" s="10"/>
-    </row>
-    <row r="6" spans="1:33" ht="60" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="D6" s="8">
-        <v>1002</v>
-      </c>
-      <c r="E6" s="11">
-        <v>38732</v>
-      </c>
-      <c r="F6" s="11">
-        <v>38776</v>
-      </c>
-      <c r="G6" s="11">
-        <v>38732</v>
-      </c>
-      <c r="H6" s="11">
-        <v>38776</v>
-      </c>
-      <c r="I6" s="11">
-        <v>38721</v>
-      </c>
-      <c r="J6" s="11">
-        <v>38802</v>
-      </c>
-      <c r="K6" s="8">
-        <v>1</v>
-      </c>
-      <c r="L6" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="M6" s="8">
-        <v>20170</v>
-      </c>
-      <c r="N6" s="8">
-        <v>50</v>
-      </c>
-      <c r="P6" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q6" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="R6" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="S6" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="T6" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="U6" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="V6" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="W6" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="AA6" s="10"/>
-      <c r="AB6" s="10"/>
-      <c r="AC6" s="10"/>
-      <c r="AD6" s="10"/>
-      <c r="AE6" s="10"/>
-      <c r="AF6" s="10"/>
-      <c r="AG6" s="10"/>
-    </row>
-    <row r="7" spans="1:33" ht="75" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D7" s="8">
-        <v>1003</v>
-      </c>
-      <c r="E7" s="9">
-        <v>38733</v>
-      </c>
-      <c r="F7" s="9">
-        <v>38795</v>
-      </c>
-      <c r="G7" s="9">
-        <v>38733</v>
-      </c>
-      <c r="H7" s="9">
-        <v>38795</v>
-      </c>
-      <c r="I7" s="9">
-        <v>38719</v>
-      </c>
-      <c r="J7" s="9">
-        <v>38795</v>
-      </c>
-      <c r="K7" s="8">
-        <v>1</v>
-      </c>
-      <c r="L7" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="M7" s="8">
-        <v>13899</v>
-      </c>
-      <c r="N7" s="8">
-        <v>68</v>
-      </c>
-      <c r="P7" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q7" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="R7" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="S7" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="T7" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="U7" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="V7" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="W7" s="8" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="8" spans="1:33" ht="60" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="D8" s="8">
-        <v>1004</v>
-      </c>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="11">
-        <v>38724</v>
-      </c>
-      <c r="J8" s="11">
-        <v>38725</v>
-      </c>
-      <c r="K8" s="8">
-        <v>1</v>
-      </c>
-      <c r="L8" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="M8" s="8">
-        <v>15159</v>
-      </c>
-      <c r="Q8" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="R8" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="S8" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="X8" s="8" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="9" spans="1:33" ht="90" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="D9" s="8">
-        <v>2001</v>
-      </c>
-      <c r="E9" s="9">
-        <v>38750</v>
-      </c>
-      <c r="F9" s="9">
-        <v>38807</v>
-      </c>
-      <c r="G9" s="9">
-        <v>38750</v>
-      </c>
-      <c r="H9" s="9">
-        <v>38807</v>
-      </c>
-      <c r="I9" s="9">
-        <v>38732</v>
-      </c>
-      <c r="J9" s="9">
-        <v>38819</v>
-      </c>
-      <c r="K9" s="8">
-        <v>2</v>
-      </c>
-      <c r="L9" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="M9" s="8">
-        <v>18437</v>
-      </c>
-      <c r="N9" s="8">
-        <v>55</v>
-      </c>
-      <c r="P9" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q9" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="R9" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="S9" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="T9" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="U9" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="V9" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="W9" s="8" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="10" spans="1:33" ht="105" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="D10" s="8">
-        <v>2002</v>
-      </c>
-      <c r="E10" s="11">
-        <v>38751</v>
-      </c>
-      <c r="F10" s="11">
-        <v>38812</v>
-      </c>
-      <c r="G10" s="11">
-        <v>38751</v>
-      </c>
-      <c r="H10" s="11">
-        <v>38812</v>
-      </c>
-      <c r="I10" s="11">
-        <v>38727</v>
-      </c>
-      <c r="J10" s="11">
-        <v>38832</v>
-      </c>
-      <c r="K10" s="8">
-        <v>2</v>
-      </c>
-      <c r="L10" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="M10" s="8">
-        <v>20580</v>
-      </c>
-      <c r="N10" s="8">
-        <v>49</v>
-      </c>
-      <c r="P10" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q10" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="R10" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="S10" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="T10" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="U10" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="V10" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="W10" s="8" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="16" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="AG16" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>